<commit_message>
Value has been changed
</commit_message>
<xml_diff>
--- a/hr-data.xlsx
+++ b/hr-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26717"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Chandoo.org\Power BI\HR Data Analysis &amp; Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/555f5755c76171bd/Desktop/HR-Analytic-Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4180418F-A064-4AF3-83E7-EEC2C11D8DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{4180418F-A064-4AF3-83E7-EEC2C11D8DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF49030C-2E32-4D1B-97B7-EB75AADA5E12}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4A559B37-D7A8-448D-91D3-7F92E46297F4}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10780" xr2:uid="{4A559B37-D7A8-448D-91D3-7F92E46297F4}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1125,7 +1125,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1413,7 +1413,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1422,20 +1422,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7278C99-611B-4334-B1D5-6B7987343580}">
   <dimension ref="A1:I162"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.8984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.78515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.92578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.0703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.8984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.92578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1519,10 +1519,10 @@
         <v>32.700000000000003</v>
       </c>
       <c r="I3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1609,7 +1609,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -1841,7 +1841,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>53</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>57</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>61</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>65</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>67</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>69</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>73</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>79</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>83</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>85</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>87</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>89</v>
       </c>
@@ -2363,7 +2363,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>91</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>93</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>95</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>97</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>99</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>101</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>103</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>105</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>107</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>109</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>112</v>
       </c>
@@ -2682,7 +2682,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>114</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>116</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>118</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>120</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>122</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>124</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>128</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>130</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>132</v>
       </c>
@@ -2972,7 +2972,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>134</v>
       </c>
@@ -3001,7 +3001,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>136</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>138</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>140</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>143</v>
       </c>
@@ -3117,7 +3117,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>145</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>147</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>149</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>152</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>154</v>
       </c>
@@ -3262,7 +3262,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>157</v>
       </c>
@@ -3291,7 +3291,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>159</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>161</v>
       </c>
@@ -3349,7 +3349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>163</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>165</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>120</v>
       </c>
@@ -3436,7 +3436,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>169</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>171</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>173</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>175</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>177</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>179</v>
       </c>
@@ -3610,7 +3610,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>181</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>183</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>185</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>187</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>189</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>191</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>194</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>196</v>
       </c>
@@ -3842,7 +3842,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>198</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>200</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>202</v>
       </c>
@@ -3929,7 +3929,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>204</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>206</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>208</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>210</v>
       </c>
@@ -4045,7 +4045,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>212</v>
       </c>
@@ -4074,7 +4074,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>214</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>216</v>
       </c>
@@ -4132,7 +4132,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>218</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>38</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>221</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>223</v>
       </c>
@@ -4248,7 +4248,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>225</v>
       </c>
@@ -4277,7 +4277,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>227</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>229</v>
       </c>
@@ -4335,7 +4335,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>231</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>151</v>
       </c>
@@ -4393,7 +4393,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>234</v>
       </c>
@@ -4422,7 +4422,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>156</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>237</v>
       </c>
@@ -4480,7 +4480,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>239</v>
       </c>
@@ -4509,7 +4509,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>111</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>52</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>243</v>
       </c>
@@ -4596,7 +4596,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>245</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>247</v>
       </c>
@@ -4654,7 +4654,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>249</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>251</v>
       </c>
@@ -4712,7 +4712,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>253</v>
       </c>
@@ -4741,7 +4741,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>255</v>
       </c>
@@ -4770,7 +4770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>257</v>
       </c>
@@ -4799,7 +4799,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>259</v>
       </c>
@@ -4828,7 +4828,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>193</v>
       </c>
@@ -4857,7 +4857,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>262</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>264</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>266</v>
       </c>
@@ -4944,7 +4944,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>268</v>
       </c>
@@ -4973,7 +4973,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>270</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>272</v>
       </c>
@@ -5031,7 +5031,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>274</v>
       </c>
@@ -5060,7 +5060,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>276</v>
       </c>
@@ -5089,7 +5089,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>278</v>
       </c>
@@ -5118,7 +5118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>28</v>
       </c>
@@ -5147,7 +5147,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>281</v>
       </c>
@@ -5176,7 +5176,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>283</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>285</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>221</v>
       </c>
@@ -5263,7 +5263,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>288</v>
       </c>
@@ -5292,7 +5292,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>290</v>
       </c>
@@ -5321,7 +5321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>292</v>
       </c>
@@ -5350,7 +5350,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>294</v>
       </c>
@@ -5379,7 +5379,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>296</v>
       </c>
@@ -5408,7 +5408,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>298</v>
       </c>
@@ -5437,7 +5437,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>300</v>
       </c>
@@ -5466,7 +5466,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>302</v>
       </c>
@@ -5495,7 +5495,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>168</v>
       </c>
@@ -5524,7 +5524,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>142</v>
       </c>
@@ -5553,7 +5553,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>306</v>
       </c>
@@ -5582,7 +5582,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>308</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>310</v>
       </c>
@@ -5640,7 +5640,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>312</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>314</v>
       </c>
@@ -5698,7 +5698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>55</v>
       </c>
@@ -5727,7 +5727,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>251</v>
       </c>
@@ -5756,7 +5756,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>318</v>
       </c>
@@ -5785,7 +5785,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>288</v>
       </c>
@@ -5814,7 +5814,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>257</v>
       </c>
@@ -5843,7 +5843,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>292</v>
       </c>
@@ -5872,7 +5872,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>294</v>
       </c>
@@ -5901,7 +5901,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>324</v>
       </c>
@@ -5930,7 +5930,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>298</v>
       </c>
@@ -5959,7 +5959,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>300</v>
       </c>
@@ -5988,7 +5988,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>328</v>
       </c>
@@ -6017,7 +6017,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>168</v>
       </c>
@@ -6046,7 +6046,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>142</v>
       </c>
@@ -6075,7 +6075,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>306</v>
       </c>
@@ -6104,7 +6104,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>308</v>
       </c>

</xml_diff>